<commit_message>
Update vehicle compatibility test to refine filtering logic and limit results
</commit_message>
<xml_diff>
--- a/src/resources/data/catalogInfo/excels/Pad_katalog_full.xlsx
+++ b/src/resources/data/catalogInfo/excels/Pad_katalog_full.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/burakarikboga/Desktop/Projects/Yavuzsan/API_SCRAPE/src/resources/data/catalogInfo/excels/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8C95B35-6593-604D-B805-2C39F298BE0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A6535B2-2273-9646-96FF-BC1E10A18D92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="35840" windowHeight="22400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="21900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
Update Excel catalog files for Crankshaft, Disc, Drum, and Pad
</commit_message>
<xml_diff>
--- a/src/resources/data/catalogInfo/excels/Pad_katalog_full.xlsx
+++ b/src/resources/data/catalogInfo/excels/Pad_katalog_full.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\URETIM9\Desktop\Projects\API_SCRAPE\src\resources\data\catalogInfo\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44483387-5CA1-4D4A-9941-8C492CD7EC2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A30DC1-578F-4340-9D50-9E952E5E8357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1884" yWindow="2652" windowWidth="20532" windowHeight="8568" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1674" uniqueCount="1600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1667" uniqueCount="1592">
   <si>
     <t>BREMBO</t>
   </si>
@@ -4648,144 +4648,48 @@
     <t>P 23 001, P 59 002</t>
   </si>
   <si>
-    <t>2039204, 2958101, 2958104, 2958106</t>
-  </si>
-  <si>
-    <t>GDB1297</t>
-  </si>
-  <si>
     <t>P 59 005, P 59 006</t>
   </si>
   <si>
     <t>P 24 029, P 24 031</t>
   </si>
   <si>
-    <t>2130501, 2130503, 2130504, 2130581, 2130591</t>
-  </si>
-  <si>
-    <t>GDB1030, GDB792</t>
-  </si>
-  <si>
-    <t>GDB3092, GDB849</t>
-  </si>
-  <si>
-    <t>GDB3051, GDB3170, GDB3368</t>
-  </si>
-  <si>
-    <t>2166404, 2166481, 2166491</t>
-  </si>
-  <si>
-    <t>GDB3101, GDB3169, GDB7521, GDB895</t>
-  </si>
-  <si>
-    <t>GDB1145, GDB3306, GDB7581</t>
-  </si>
-  <si>
-    <t>2213801, 2213901</t>
-  </si>
-  <si>
-    <t>2301802, 2301881, 2301891</t>
-  </si>
-  <si>
-    <t>2307801, 2307881, 2307891</t>
-  </si>
-  <si>
     <t>P 68 024, P 68 024X, P 68 035</t>
   </si>
   <si>
-    <t>2355405, 2355406</t>
-  </si>
-  <si>
     <t>P 85 020, P 85 020X, P 85 089</t>
   </si>
   <si>
-    <t>GDB1055, GDB1196, GDB1267, GDB1311, GDB1330, GDB1372, GDB1438, GDB1458, GDB1504, GDB2040, GDB7612</t>
-  </si>
-  <si>
     <t>P 06 037, P 06 037X, P 06 37X</t>
   </si>
   <si>
-    <t>GDB4126, GDB7627</t>
-  </si>
-  <si>
     <t>P 23 085, P 23 108, P 23 140, P 23 202, P 23 202N</t>
   </si>
   <si>
     <t>P 23 089, P 23 109, P 23 111, P 23 199</t>
   </si>
   <si>
-    <t>2119303, 2219301, 2377501</t>
-  </si>
-  <si>
     <t>P 85 084, P 85 086, P 85 097</t>
   </si>
   <si>
-    <t>2376302, 2376381, 2395001, 2395081, 2395091</t>
-  </si>
-  <si>
     <t>P 30 034, P 30 034X, P 30 077, P 30 162, P 30 162N</t>
   </si>
   <si>
-    <t>2396601, 2396605, 2396606</t>
-  </si>
-  <si>
     <t>P 65 014, P 65 015, P 65 015N</t>
   </si>
   <si>
-    <t>2404901, 2404902, 2404903</t>
-  </si>
-  <si>
     <t>P 06 058, P 06 058N</t>
   </si>
   <si>
-    <t>2428301, 2428302</t>
-  </si>
-  <si>
     <t>P 85 112, P 85 112X, P 85 130, P 85 130N, P 85 130X</t>
   </si>
   <si>
-    <t>GDB7738</t>
-  </si>
-  <si>
     <t>P 23 104, P 59 047, P 59 057</t>
   </si>
   <si>
     <t>P 06 073, P 06 115</t>
   </si>
   <si>
-    <t>2443801, 2443901, 2443903</t>
-  </si>
-  <si>
-    <t>2448301, 2448302, 2448305, 2448381, 2448382, 2448391, 2448392</t>
-  </si>
-  <si>
-    <t>2456101, 2456102, 2456103, 2456181</t>
-  </si>
-  <si>
-    <t>2459501, 2459502</t>
-  </si>
-  <si>
-    <t>GDB3577, GDB7238, GDB7743</t>
-  </si>
-  <si>
-    <t>2470501, 2470601, 2470681</t>
-  </si>
-  <si>
-    <t>2473801, 2473803, 2473805, 2473808</t>
-  </si>
-  <si>
-    <t>2426401, 2440801</t>
-  </si>
-  <si>
-    <t>2460605, 2521401, 2521404, 2521405</t>
-  </si>
-  <si>
-    <t>GDB3549, GDB7845</t>
-  </si>
-  <si>
-    <t>2917270, 2919201, 2919202, 2919209</t>
-  </si>
-  <si>
     <t>2167904, 2167907</t>
   </si>
   <si>
@@ -4832,6 +4736,78 @@
   </si>
   <si>
     <t>P 61 127, P 61 127X</t>
+  </si>
+  <si>
+    <t>GDB1030</t>
+  </si>
+  <si>
+    <t>GDB3092</t>
+  </si>
+  <si>
+    <t>GDB3170, GDB3368</t>
+  </si>
+  <si>
+    <t>GDB3101, GDB3169, GDB895</t>
+  </si>
+  <si>
+    <t>GDB1145, GDB3306</t>
+  </si>
+  <si>
+    <t>GDB1055, GDB1196, GDB1267, GDB1311, GDB1330, GDB1372, GDB1438, GDB1458, GDB1504, GDB2040</t>
+  </si>
+  <si>
+    <t>GDB4126</t>
+  </si>
+  <si>
+    <t>GDB3577</t>
+  </si>
+  <si>
+    <t>GDB3549</t>
+  </si>
+  <si>
+    <t>2919201, 2919202, 2919209</t>
+  </si>
+  <si>
+    <t>2521401, 2521404, 2521405</t>
+  </si>
+  <si>
+    <t>2473801, 2473803, 2473805</t>
+  </si>
+  <si>
+    <t>2470601, 2470681</t>
+  </si>
+  <si>
+    <t>2456101, 2456103, 2456181</t>
+  </si>
+  <si>
+    <t>2448301, 2448302, 2448305, 2448381, 2448382</t>
+  </si>
+  <si>
+    <t>2404901, 2404903</t>
+  </si>
+  <si>
+    <t>2396601, 2396605</t>
+  </si>
+  <si>
+    <t>2376302, 2376381, 2395001, 2395081</t>
+  </si>
+  <si>
+    <t>2119303, 2377501</t>
+  </si>
+  <si>
+    <t>2307801, 2307881</t>
+  </si>
+  <si>
+    <t>2301802, 2301881</t>
+  </si>
+  <si>
+    <t>2166404, 2166481</t>
+  </si>
+  <si>
+    <t>2130501, 2130503, 2130504, 2130581</t>
+  </si>
+  <si>
+    <t>2039204, 2958101, 2958104</t>
   </si>
 </sst>
 </file>
@@ -5481,7 +5457,7 @@
         <v>562</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>1538</v>
+        <v>1591</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>16</v>
@@ -5653,9 +5629,7 @@
       <c r="D20" s="3" t="s">
         <v>561</v>
       </c>
-      <c r="E20" s="3" t="s">
-        <v>1539</v>
-      </c>
+      <c r="E20" s="3"/>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="3">
@@ -5750,7 +5724,7 @@
         <v>180454</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>1540</v>
+        <v>1538</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>1311</v>
@@ -5971,7 +5945,7 @@
         <v>180790</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>1541</v>
+        <v>1539</v>
       </c>
       <c r="D39" s="3">
         <v>2117105</v>
@@ -6110,7 +6084,7 @@
         <v>602</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>1542</v>
+        <v>1590</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>49</v>
@@ -6266,7 +6240,7 @@
         <v>2138802</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>1543</v>
+        <v>1568</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -6521,7 +6495,7 @@
         <v>2154501</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>1544</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -6555,7 +6529,7 @@
         <v>2155301</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>1545</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -6720,7 +6694,7 @@
         <v>645</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>1546</v>
+        <v>1589</v>
       </c>
       <c r="E83" s="3" t="s">
         <v>79</v>
@@ -6786,7 +6760,7 @@
         <v>650</v>
       </c>
       <c r="D87" s="9" t="s">
-        <v>1584</v>
+        <v>1552</v>
       </c>
       <c r="E87" s="3" t="s">
         <v>83</v>
@@ -6891,7 +6865,7 @@
         <v>1329</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>1547</v>
+        <v>1571</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -7248,7 +7222,7 @@
         <v>2196102</v>
       </c>
       <c r="E114" s="3" t="s">
-        <v>1548</v>
+        <v>1572</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -7550,8 +7524,8 @@
       <c r="C132" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="D132" s="3" t="s">
-        <v>1549</v>
+      <c r="D132" s="3">
+        <v>2213901</v>
       </c>
       <c r="E132" s="3" t="s">
         <v>561</v>
@@ -8551,10 +8525,10 @@
         <v>181331</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>1585</v>
+        <v>1553</v>
       </c>
       <c r="D191" s="3" t="s">
-        <v>1550</v>
+        <v>1588</v>
       </c>
       <c r="E191" s="3" t="s">
         <v>774</v>
@@ -8707,7 +8681,7 @@
         <v>783</v>
       </c>
       <c r="D200" s="3" t="s">
-        <v>1551</v>
+        <v>1587</v>
       </c>
       <c r="E200" s="3" t="s">
         <v>165</v>
@@ -8891,7 +8865,7 @@
         <v>181349</v>
       </c>
       <c r="C211" s="10" t="s">
-        <v>1586</v>
+        <v>1554</v>
       </c>
       <c r="D211" s="3" t="s">
         <v>1349</v>
@@ -8908,7 +8882,7 @@
         <v>179</v>
       </c>
       <c r="C212" s="3" t="s">
-        <v>1587</v>
+        <v>1555</v>
       </c>
       <c r="D212" s="3" t="s">
         <v>1350</v>
@@ -9397,7 +9371,7 @@
         <v>181577</v>
       </c>
       <c r="C241" s="10" t="s">
-        <v>1588</v>
+        <v>1556</v>
       </c>
       <c r="D241" s="3" t="s">
         <v>1357</v>
@@ -9618,7 +9592,7 @@
         <v>227</v>
       </c>
       <c r="C254" s="3" t="s">
-        <v>1589</v>
+        <v>1557</v>
       </c>
       <c r="D254" s="3" t="s">
         <v>1361</v>
@@ -9924,7 +9898,7 @@
         <v>181962</v>
       </c>
       <c r="C272" s="3" t="s">
-        <v>1590</v>
+        <v>1558</v>
       </c>
       <c r="D272" s="3" t="s">
         <v>1366</v>
@@ -10094,10 +10068,10 @@
         <v>250</v>
       </c>
       <c r="C282" s="3" t="s">
-        <v>1552</v>
-      </c>
-      <c r="D282" s="3" t="s">
-        <v>1553</v>
+        <v>1540</v>
+      </c>
+      <c r="D282" s="3">
+        <v>2355406</v>
       </c>
       <c r="E282" s="3" t="s">
         <v>883</v>
@@ -10111,13 +10085,13 @@
         <v>251</v>
       </c>
       <c r="C283" s="3" t="s">
-        <v>1554</v>
+        <v>1541</v>
       </c>
       <c r="D283" s="3" t="s">
         <v>1373</v>
       </c>
       <c r="E283" s="3" t="s">
-        <v>1555</v>
+        <v>1573</v>
       </c>
     </row>
     <row r="284" spans="1:5">
@@ -10228,7 +10202,7 @@
         <v>181806</v>
       </c>
       <c r="C290" s="3" t="s">
-        <v>1591</v>
+        <v>1559</v>
       </c>
       <c r="D290" s="3" t="s">
         <v>1377</v>
@@ -10381,7 +10355,7 @@
         <v>269</v>
       </c>
       <c r="C299" s="3" t="s">
-        <v>1556</v>
+        <v>1542</v>
       </c>
       <c r="D299" s="3" t="s">
         <v>1381</v>
@@ -10404,7 +10378,7 @@
         <v>2363801</v>
       </c>
       <c r="E300" s="3" t="s">
-        <v>1557</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="301" spans="1:5">
@@ -10602,7 +10576,7 @@
         <v>277</v>
       </c>
       <c r="C312" s="3" t="s">
-        <v>1558</v>
+        <v>1543</v>
       </c>
       <c r="D312" s="3" t="s">
         <v>1389</v>
@@ -10959,7 +10933,7 @@
         <v>181780</v>
       </c>
       <c r="C333" s="3" t="s">
-        <v>1559</v>
+        <v>1544</v>
       </c>
       <c r="D333" s="3" t="s">
         <v>1401</v>
@@ -11028,7 +11002,7 @@
       </c>
       <c r="C337" s="8"/>
       <c r="D337" s="3" t="s">
-        <v>1560</v>
+        <v>1586</v>
       </c>
       <c r="E337" s="3" t="s">
         <v>949</v>
@@ -11567,10 +11541,10 @@
         <v>181654</v>
       </c>
       <c r="C369" s="3" t="s">
-        <v>1561</v>
+        <v>1545</v>
       </c>
       <c r="D369" s="3" t="s">
-        <v>1562</v>
+        <v>1585</v>
       </c>
       <c r="E369" s="3" t="s">
         <v>991</v>
@@ -11652,10 +11626,10 @@
         <v>181540</v>
       </c>
       <c r="C374" s="3" t="s">
-        <v>1563</v>
+        <v>1546</v>
       </c>
       <c r="D374" s="3" t="s">
-        <v>1564</v>
+        <v>1584</v>
       </c>
       <c r="E374" s="3" t="s">
         <v>997</v>
@@ -11924,10 +11898,10 @@
         <v>182204</v>
       </c>
       <c r="C390" s="3" t="s">
-        <v>1565</v>
+        <v>1547</v>
       </c>
       <c r="D390" s="3" t="s">
-        <v>1566</v>
+        <v>1583</v>
       </c>
       <c r="E390" s="3" t="s">
         <v>354</v>
@@ -12332,7 +12306,7 @@
         <v>181905</v>
       </c>
       <c r="C414" s="3" t="s">
-        <v>1567</v>
+        <v>1548</v>
       </c>
       <c r="D414" s="3">
         <v>2417201</v>
@@ -12572,8 +12546,8 @@
       <c r="C428" s="3" t="s">
         <v>1057</v>
       </c>
-      <c r="D428" s="3" t="s">
-        <v>1568</v>
+      <c r="D428" s="3">
+        <v>2428302</v>
       </c>
       <c r="E428" s="3" t="s">
         <v>1058</v>
@@ -12740,7 +12714,7 @@
         <v>181923</v>
       </c>
       <c r="C438" s="3" t="s">
-        <v>1569</v>
+        <v>1549</v>
       </c>
       <c r="D438" s="3" t="s">
         <v>1448</v>
@@ -12813,9 +12787,7 @@
       <c r="D442" s="3" t="s">
         <v>1451</v>
       </c>
-      <c r="E442" s="3" t="s">
-        <v>1570</v>
-      </c>
+      <c r="E442" s="3"/>
     </row>
     <row r="443" spans="1:5">
       <c r="A443" s="3">
@@ -12825,7 +12797,7 @@
         <v>399</v>
       </c>
       <c r="C443" s="3" t="s">
-        <v>1571</v>
+        <v>1550</v>
       </c>
       <c r="D443" s="3" t="s">
         <v>1452</v>
@@ -12876,7 +12848,7 @@
         <v>141816</v>
       </c>
       <c r="C446" s="4" t="s">
-        <v>1592</v>
+        <v>1560</v>
       </c>
       <c r="D446" s="3">
         <v>2436803</v>
@@ -13029,7 +13001,7 @@
         <v>181992</v>
       </c>
       <c r="C455" s="3" t="s">
-        <v>1572</v>
+        <v>1551</v>
       </c>
       <c r="D455" s="3" t="s">
         <v>1456</v>
@@ -13048,8 +13020,8 @@
       <c r="C456" s="3" t="s">
         <v>1087</v>
       </c>
-      <c r="D456" s="3" t="s">
-        <v>1573</v>
+      <c r="D456" s="3">
+        <v>2443901</v>
       </c>
       <c r="E456" s="3" t="s">
         <v>414</v>
@@ -13114,7 +13086,7 @@
         <v>141836</v>
       </c>
       <c r="C460" s="10" t="s">
-        <v>1593</v>
+        <v>1561</v>
       </c>
       <c r="D460" s="3" t="s">
         <v>1458</v>
@@ -13185,7 +13157,7 @@
         <v>1095</v>
       </c>
       <c r="D464" s="3" t="s">
-        <v>1574</v>
+        <v>1582</v>
       </c>
       <c r="E464" s="3" t="s">
         <v>422</v>
@@ -13540,7 +13512,7 @@
         <v>1123</v>
       </c>
       <c r="D485" s="3" t="s">
-        <v>1575</v>
+        <v>1581</v>
       </c>
       <c r="E485" s="3" t="s">
         <v>1124</v>
@@ -13607,8 +13579,8 @@
       <c r="C489" s="3" t="s">
         <v>1128</v>
       </c>
-      <c r="D489" s="3" t="s">
-        <v>1576</v>
+      <c r="D489" s="3">
+        <v>2459501</v>
       </c>
       <c r="E489" s="3" t="s">
         <v>1129</v>
@@ -13798,7 +13770,7 @@
         <v>2468201</v>
       </c>
       <c r="E500" s="3" t="s">
-        <v>1577</v>
+        <v>1575</v>
       </c>
     </row>
     <row r="501" spans="1:5">
@@ -13931,7 +13903,7 @@
         <v>1152</v>
       </c>
       <c r="D508" s="3" t="s">
-        <v>1578</v>
+        <v>1580</v>
       </c>
       <c r="E508" s="3" t="s">
         <v>452</v>
@@ -14081,9 +14053,7 @@
       <c r="C517" s="3" t="s">
         <v>1164</v>
       </c>
-      <c r="D517" s="3" t="s">
-        <v>1580</v>
-      </c>
+      <c r="D517" s="3"/>
       <c r="E517" s="3" t="s">
         <v>1165</v>
       </c>
@@ -14317,7 +14287,7 @@
         <v>181928</v>
       </c>
       <c r="C531" s="3" t="s">
-        <v>1594</v>
+        <v>1562</v>
       </c>
       <c r="D531" s="3" t="s">
         <v>1485</v>
@@ -14572,7 +14542,7 @@
         <v>181943</v>
       </c>
       <c r="C546" s="3" t="s">
-        <v>1595</v>
+        <v>1563</v>
       </c>
       <c r="D546" s="3" t="s">
         <v>1495</v>
@@ -14589,7 +14559,7 @@
         <v>182152</v>
       </c>
       <c r="C547" s="3" t="s">
-        <v>1596</v>
+        <v>1564</v>
       </c>
       <c r="D547" s="3" t="s">
         <v>1496</v>
@@ -14625,9 +14595,7 @@
       <c r="C549" s="3" t="s">
         <v>1198</v>
       </c>
-      <c r="D549" s="3">
-        <v>2511901</v>
-      </c>
+      <c r="D549" s="3"/>
       <c r="E549" s="3" t="s">
         <v>487</v>
       </c>
@@ -14898,7 +14866,7 @@
         <v>1218</v>
       </c>
       <c r="D565" s="3" t="s">
-        <v>1581</v>
+        <v>1578</v>
       </c>
       <c r="E565" s="3" t="s">
         <v>1219</v>
@@ -14946,7 +14914,7 @@
         <v>182042</v>
       </c>
       <c r="C568" s="9" t="s">
-        <v>1597</v>
+        <v>1565</v>
       </c>
       <c r="D568" s="3" t="s">
         <v>1507</v>
@@ -15371,7 +15339,7 @@
         <v>519</v>
       </c>
       <c r="C593" s="3" t="s">
-        <v>1598</v>
+        <v>1566</v>
       </c>
       <c r="D593" s="3">
         <v>2568303</v>
@@ -15445,7 +15413,7 @@
         <v>2575701</v>
       </c>
       <c r="E597" s="3" t="s">
-        <v>1582</v>
+        <v>1576</v>
       </c>
     </row>
     <row r="598" spans="1:5">
@@ -15507,7 +15475,7 @@
         <v>182166</v>
       </c>
       <c r="C601" s="3" t="s">
-        <v>1599</v>
+        <v>1567</v>
       </c>
       <c r="D601" s="3" t="s">
         <v>1517</v>
@@ -15969,7 +15937,7 @@
         <v>1287</v>
       </c>
       <c r="D628" s="3" t="s">
-        <v>1583</v>
+        <v>1577</v>
       </c>
       <c r="E628" s="3" t="s">
         <v>546</v>

</xml_diff>

<commit_message>
feat: Update Pad_katalog_full.xlsx with new data
</commit_message>
<xml_diff>
--- a/src/resources/data/catalogInfo/excels/Pad_katalog_full.xlsx
+++ b/src/resources/data/catalogInfo/excels/Pad_katalog_full.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\URETIM9\Desktop\Projects\API_SCRAPE\src\resources\data\catalogInfo\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A6CF8D6-9209-4DF5-A545-11D3C05332A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C0543F-2D19-4489-881C-3BCE0E526BDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7580,7 +7580,8 @@
     <col min="3" max="3" width="21.5546875" style="2" customWidth="1"/>
     <col min="4" max="4" width="15.109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="14" style="2" customWidth="1"/>
-    <col min="6" max="16384" width="11.5546875" style="2"/>
+    <col min="6" max="6" width="16.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="11.5546875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.6">

</xml_diff>

<commit_message>
feat: Add BREMBO product reference for P 68 029 to referenceArray
</commit_message>
<xml_diff>
--- a/src/resources/data/catalogInfo/excels/Pad_katalog_full.xlsx
+++ b/src/resources/data/catalogInfo/excels/Pad_katalog_full.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24326"/>
   <workbookPr codeName="BuÇalışmaKitabı" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\URETIM9\Desktop\Projects\API_SCRAPE\src\resources\data\catalogInfo\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C0543F-2D19-4489-881C-3BCE0E526BDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD7336A-C8BA-4AA4-BEBD-CF602329F86C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1416" yWindow="2448" windowWidth="20532" windowHeight="10140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2338" uniqueCount="2227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2341" uniqueCount="2230">
   <si>
     <t>BREMBO</t>
   </si>
@@ -7066,12 +7066,21 @@
   <si>
     <t>34211160533</t>
   </si>
+  <si>
+    <t>P 68 029</t>
+  </si>
+  <si>
+    <t>GDB1540, GDB1540DTE</t>
+  </si>
+  <si>
+    <t>410600012R</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -7171,6 +7180,13 @@
       <charset val="162"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -7201,8 +7217,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -7258,8 +7275,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{569EE802-C990-4233-A30E-A95773FD33CF}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -7572,7 +7590,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE0BEB64-BBB8-0049-A89F-86BCC9CE0A4C}">
   <sheetPr codeName="Sayfa1"/>
-  <dimension ref="A1:F638"/>
+  <dimension ref="A1:F639"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="9.44140625" style="2" bestFit="1" customWidth="1"/>
@@ -20316,6 +20334,26 @@
       </c>
       <c r="F638" s="2" t="s">
         <v>2105</v>
+      </c>
+    </row>
+    <row r="639" spans="1:6">
+      <c r="A639" s="17">
+        <v>23215208</v>
+      </c>
+      <c r="B639" s="17">
+        <v>181431</v>
+      </c>
+      <c r="C639" s="17" t="s">
+        <v>2227</v>
+      </c>
+      <c r="D639" s="17">
+        <v>2321502</v>
+      </c>
+      <c r="E639" s="17" t="s">
+        <v>2228</v>
+      </c>
+      <c r="F639" s="2" t="s">
+        <v>2229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RE-ARRANGED and made them ready to export in to Filemaker
</commit_message>
<xml_diff>
--- a/src/resources/data/catalogInfo/excels/Pad_katalog_full.xlsx
+++ b/src/resources/data/catalogInfo/excels/Pad_katalog_full.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\URETIM9\Desktop\Projects\API_SCRAPE\src\resources\data\catalogInfo\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD7336A-C8BA-4AA4-BEBD-CF602329F86C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F21044-212E-4279-811C-C752F41F434F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1416" yWindow="2448" windowWidth="20532" windowHeight="10140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="804" yWindow="1080" windowWidth="20532" windowHeight="10140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2341" uniqueCount="2230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2327" uniqueCount="2230">
   <si>
     <t>BREMBO</t>
   </si>
@@ -7221,7 +7221,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -7273,6 +7273,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -20366,222 +20369,204 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68835513-6EFD-439F-BF85-C50C0DA8007D}">
   <sheetPr codeName="Sayfa2"/>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="9" style="16" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.33203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5546875" style="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.5546875" style="16" bestFit="1" customWidth="1"/>
     <col min="4" max="16384" width="8.88671875" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="16">
+    <row r="1" spans="1:2" s="18" customFormat="1">
+      <c r="A1" s="18" t="s">
+        <v>1324</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="16">
         <v>20341401</v>
       </c>
-      <c r="B1" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C1" s="16">
+      <c r="B2" s="16">
         <v>180324</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="16">
+    <row r="3" spans="1:2">
+      <c r="A3" s="16">
         <v>21201201</v>
       </c>
-      <c r="B2" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C2" s="16">
+      <c r="B3" s="16">
         <v>181366</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="16">
+    <row r="4" spans="1:2">
+      <c r="A4" s="16">
         <v>21312201</v>
       </c>
-      <c r="B3" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C3" s="16" t="s">
+      <c r="B4" s="16" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="16">
+    <row r="5" spans="1:2">
+      <c r="A5" s="16">
         <v>21347201</v>
       </c>
-      <c r="B4" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C4" s="16">
+      <c r="B5" s="16">
         <v>140884</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="16">
+    <row r="6" spans="1:2">
+      <c r="A6" s="16">
         <v>21576201</v>
       </c>
-      <c r="B5" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C5" s="16" t="s">
+      <c r="B6" s="16" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="16">
+    <row r="7" spans="1:2">
+      <c r="A7" s="16">
         <v>21621201</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C6" s="16">
+      <c r="B7" s="16">
         <v>141102</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="16">
+    <row r="8" spans="1:2">
+      <c r="A8" s="16">
         <v>21857201</v>
       </c>
-      <c r="B7" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C7" s="16">
+      <c r="B8" s="16">
         <v>181150</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="16">
+    <row r="9" spans="1:2">
+      <c r="A9" s="16">
         <v>22531201</v>
       </c>
-      <c r="B8" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C8" s="16" t="s">
+      <c r="B9" s="16" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="16">
+    <row r="10" spans="1:2">
+      <c r="A10" s="16">
         <v>23177401</v>
       </c>
-      <c r="B9" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C9" s="16" t="s">
+      <c r="B10" s="16" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="16">
+    <row r="11" spans="1:2">
+      <c r="A11" s="16">
         <v>23258108</v>
       </c>
-      <c r="B10" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C10" s="16" t="s">
+      <c r="B11" s="16" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="16">
-        <v>23279401</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C11" s="16">
-        <v>180801</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:2">
       <c r="A12" s="16">
+        <v>23510101</v>
+      </c>
+      <c r="B12" s="16">
+        <v>181583</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="16">
         <v>23554410</v>
       </c>
-      <c r="B12" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C12" s="16" t="s">
+      <c r="B13" s="16" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
-      <c r="A13" s="16">
+    <row r="14" spans="1:2">
+      <c r="A14" s="16">
         <v>23775201</v>
       </c>
-      <c r="B13" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C13" s="16">
+      <c r="B14" s="16">
         <v>181596</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="16">
+    <row r="15" spans="1:2">
+      <c r="A15" s="16">
         <v>23901206</v>
       </c>
-      <c r="B14" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C14" s="16">
+      <c r="B15" s="16">
         <v>141103</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="16">
+    <row r="16" spans="1:2">
+      <c r="A16" s="16">
         <v>24072401</v>
       </c>
-      <c r="B15" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C15" s="16">
+      <c r="B16" s="16">
         <v>181659</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
-      <c r="A16" s="16">
+    <row r="17" spans="1:2">
+      <c r="A17" s="16">
         <v>24073303</v>
       </c>
-      <c r="B16" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C16" s="16">
+      <c r="B17" s="16">
         <v>181845</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="16">
+    <row r="18" spans="1:2">
+      <c r="A18" s="16">
         <v>24073401</v>
       </c>
-      <c r="B17" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C17" s="16" t="s">
+      <c r="B18" s="16" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="16">
+    <row r="19" spans="1:2">
+      <c r="A19" s="16">
         <v>24498201</v>
       </c>
-      <c r="B18" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C18" s="16">
+      <c r="B19" s="16">
         <v>181799</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="16">
+    <row r="20" spans="1:2">
+      <c r="A20" s="16">
         <v>24510201</v>
       </c>
-      <c r="B19" s="16" t="s">
-        <v>555</v>
-      </c>
-      <c r="C19" s="16">
+      <c r="B20" s="16">
         <v>181798</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="16">
+        <v>24710201</v>
+      </c>
+      <c r="B21" s="16">
+        <v>181856</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="16">
+        <v>24883401</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="16">
+        <v>26188208</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="16">
+        <v>29153401</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>545</v>
       </c>
     </row>
   </sheetData>

</xml_diff>